<commit_message>
Day 5: Fix Formspree AJAX submission and complete portfolio personalization
</commit_message>
<xml_diff>
--- a/Standalone_Daily_Progress_Tracker.xlsx
+++ b/Standalone_Daily_Progress_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\web-dev-journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5837C7D6-CE7B-404A-8CC0-5EE2C029F831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2E0DB11-3000-47D5-8220-B894F7416D66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1902" yWindow="1902" windowWidth="19562" windowHeight="10161" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Progress Log" sheetId="1" r:id="rId1"/>
@@ -436,9 +436,50 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{5A2139C3-C532-4997-AC2B-31B6DA1BF1F9}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{CA5E5F3B-9941-4707-91D2-83BCD520B1DF}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -737,7 +778,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="94" customWidth="1"/>
     <col min="2" max="3" width="14" customWidth="1"/>
@@ -752,17 +793,17 @@
     <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="21.1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -782,10 +823,10 @@
       </c>
       <c r="H4" s="6">
         <f>COUNTIF(L8:L37, "Completed")/COUNTA(A8:A37)</f>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>5</v>
       </c>
@@ -823,7 +864,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>17</v>
       </c>
@@ -862,7 +903,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>23</v>
       </c>
@@ -901,7 +942,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>25</v>
       </c>
@@ -940,7 +981,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>27</v>
       </c>
@@ -976,10 +1017,10 @@
         <v>21</v>
       </c>
       <c r="L11" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>30</v>
       </c>
@@ -1015,10 +1056,10 @@
         <v>21</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>32</v>
       </c>
@@ -1057,7 +1098,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>34</v>
       </c>
@@ -1095,7 +1136,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>40</v>
       </c>
@@ -1134,7 +1175,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>42</v>
       </c>
@@ -1173,7 +1214,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>43</v>
       </c>
@@ -1212,7 +1253,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>44</v>
       </c>
@@ -1251,7 +1292,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>45</v>
       </c>
@@ -1290,7 +1331,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>46</v>
       </c>
@@ -1329,7 +1370,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>47</v>
       </c>
@@ -1367,7 +1408,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>48</v>
       </c>
@@ -1406,7 +1447,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>50</v>
       </c>
@@ -1445,7 +1486,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>51</v>
       </c>
@@ -1484,7 +1525,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>52</v>
       </c>
@@ -1523,7 +1564,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>53</v>
       </c>
@@ -1562,7 +1603,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>54</v>
       </c>
@@ -1601,7 +1642,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>55</v>
       </c>
@@ -1639,7 +1680,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>56</v>
       </c>
@@ -1678,7 +1719,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>57</v>
       </c>
@@ -1717,7 +1758,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>58</v>
       </c>
@@ -1756,7 +1797,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>59</v>
       </c>
@@ -1795,7 +1836,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>60</v>
       </c>
@@ -1834,7 +1875,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>61</v>
       </c>
@@ -1873,7 +1914,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>62</v>
       </c>
@@ -1911,7 +1952,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>63</v>
       </c>
@@ -1950,7 +1991,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>64</v>
       </c>
@@ -1990,6 +2031,25 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="L8:L37">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Rest Day">
+      <formula>NOT(ISERROR(SEARCH("Rest Day",L8)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",L8)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="In Progress">
+      <formula>NOT(ISERROR(SEARCH("In Progress",L8)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Completed">
+      <formula>NOT(ISERROR(SEARCH("Completed",L8)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid Entry" error="Your entry is not in the list" promptTitle="Select Status" prompt="Please select from the list" sqref="L8:L100" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"Pending,Completed,In Progress,Rest Day"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1997,7 +2057,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -2008,17 +2068,17 @@
     <col min="7" max="7" width="43" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="21.1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>67</v>
       </c>
@@ -2041,7 +2101,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>74</v>
       </c>
@@ -2067,7 +2127,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>76</v>
       </c>
@@ -2093,7 +2153,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>78</v>
       </c>
@@ -2119,7 +2179,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>80</v>
       </c>

</xml_diff>

<commit_message>
Day 6 Complete Smart Expense Tracker app and wrap Phase 1
</commit_message>
<xml_diff>
--- a/Standalone_Daily_Progress_Tracker.xlsx
+++ b/Standalone_Daily_Progress_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\web-dev-journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2E0DB11-3000-47D5-8220-B894F7416D66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBED65EF-91F4-455B-8DCB-C4AA0CAABA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1902" yWindow="1902" windowWidth="19562" windowHeight="10161" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -823,7 +823,7 @@
       </c>
       <c r="H4" s="6">
         <f>COUNTIF(L8:L37, "Completed")/COUNTA(A8:A37)</f>
-        <v>0.16666666666666666</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1095,7 +1095,7 @@
         <v>21</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1172,7 +1172,7 @@
         <v>21</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -1211,7 +1211,7 @@
         <v>21</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -1250,7 +1250,7 @@
         <v>21</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -1289,7 +1289,7 @@
         <v>21</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -1328,7 +1328,7 @@
         <v>21</v>
       </c>
       <c r="L19" s="11" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -1367,7 +1367,7 @@
         <v>21</v>
       </c>
       <c r="L20" s="11" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>